<commit_message>
Refine OG0044 quiz answers
</commit_message>
<xml_diff>
--- a/v3/OG0044/OG0044_DevSpec.xlsx
+++ b/v3/OG0044/OG0044_DevSpec.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METADATA" sheetId="1" r:id="Rd24c2780afd54682"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUESTION_SPEC" sheetId="2" r:id="R1f5c74f29bd2444b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASSETS" sheetId="3" r:id="Rb54e93a8d59740a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESPONSE_QUALITY" sheetId="4" r:id="Rb313bdb113794c51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METADATA" sheetId="1" r:id="R6a5318c23fcf4d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUESTION_SPEC" sheetId="2" r:id="R84be0c6d2ae44cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASSETS" sheetId="3" r:id="R3e5af636cf3d465f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESPONSE_QUALITY" sheetId="4" r:id="Re5bba7a474ab4bb2"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>